<commit_message>
update math model: S32 strips, 10 paylines, new bonus pools
- Reel strips redesigned to 32 positions with new symbol distribution
- Paylines reduced from 20 to 10
- Bonus prize pools updated (225/300/300x), buy bonus limited to tier 1-2
- GDD rewritten in English with updated values
- Excel regenerated to match new math

via [Happy](https://happy.engineering)
</commit_message>
<xml_diff>
--- a/docs/total-bet-model-rtp.xlsx
+++ b/docs/total-bet-model-rtp.xlsx
@@ -85,9 +85,9 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:U67"/>
+  <dimension ref="B2:U71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -519,10 +519,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F3" s="2">
         <f>D3^B3</f>
@@ -618,23 +618,23 @@
         </is>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIF(B$19:B$38,$B6)</f>
+        <f>COUNTIF(B$19:B$50,$B6)</f>
         <v/>
       </c>
       <c r="D6" s="2">
-        <f>COUNTIF(C$19:C$38,$B6)</f>
+        <f>COUNTIF(C$19:C$50,$B6)</f>
         <v/>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIF(D$19:D$38,$B6)</f>
+        <f>COUNTIF(D$19:D$50,$B6)</f>
         <v/>
       </c>
       <c r="F6" s="2">
-        <f>COUNTIF(E$19:E$38,$B6)</f>
+        <f>COUNTIF(E$19:E$50,$B6)</f>
         <v/>
       </c>
       <c r="G6" s="2">
-        <f>COUNTIF(F$19:F$38,$B6)</f>
+        <f>COUNTIF(F$19:F$50,$B6)</f>
         <v/>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -686,23 +686,23 @@
         </is>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIF(B$19:B$38,$B7)</f>
+        <f>COUNTIF(B$19:B$50,$B7)</f>
         <v/>
       </c>
       <c r="D7" s="2">
-        <f>COUNTIF(C$19:C$38,$B7)</f>
+        <f>COUNTIF(C$19:C$50,$B7)</f>
         <v/>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIF(D$19:D$38,$B7)</f>
+        <f>COUNTIF(D$19:D$50,$B7)</f>
         <v/>
       </c>
       <c r="F7" s="2">
-        <f>COUNTIF(E$19:E$38,$B7)</f>
+        <f>COUNTIF(E$19:E$50,$B7)</f>
         <v/>
       </c>
       <c r="G7" s="2">
-        <f>COUNTIF(F$19:F$38,$B7)</f>
+        <f>COUNTIF(F$19:F$50,$B7)</f>
         <v/>
       </c>
       <c r="I7" s="1" t="inlineStr">
@@ -754,23 +754,23 @@
         </is>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIF(B$19:B$38,$B8)</f>
+        <f>COUNTIF(B$19:B$50,$B8)</f>
         <v/>
       </c>
       <c r="D8" s="2">
-        <f>COUNTIF(C$19:C$38,$B8)</f>
+        <f>COUNTIF(C$19:C$50,$B8)</f>
         <v/>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIF(D$19:D$38,$B8)</f>
+        <f>COUNTIF(D$19:D$50,$B8)</f>
         <v/>
       </c>
       <c r="F8" s="2">
-        <f>COUNTIF(E$19:E$38,$B8)</f>
+        <f>COUNTIF(E$19:E$50,$B8)</f>
         <v/>
       </c>
       <c r="G8" s="2">
-        <f>COUNTIF(F$19:F$38,$B8)</f>
+        <f>COUNTIF(F$19:F$50,$B8)</f>
         <v/>
       </c>
       <c r="I8" s="1" t="inlineStr">
@@ -822,23 +822,23 @@
         </is>
       </c>
       <c r="C9" s="2">
-        <f>COUNTIF(B$19:B$38,$B9)</f>
+        <f>COUNTIF(B$19:B$50,$B9)</f>
         <v/>
       </c>
       <c r="D9" s="2">
-        <f>COUNTIF(C$19:C$38,$B9)</f>
+        <f>COUNTIF(C$19:C$50,$B9)</f>
         <v/>
       </c>
       <c r="E9" s="2">
-        <f>COUNTIF(D$19:D$38,$B9)</f>
+        <f>COUNTIF(D$19:D$50,$B9)</f>
         <v/>
       </c>
       <c r="F9" s="2">
-        <f>COUNTIF(E$19:E$38,$B9)</f>
+        <f>COUNTIF(E$19:E$50,$B9)</f>
         <v/>
       </c>
       <c r="G9" s="2">
-        <f>COUNTIF(F$19:F$38,$B9)</f>
+        <f>COUNTIF(F$19:F$50,$B9)</f>
         <v/>
       </c>
       <c r="I9" s="1" t="inlineStr">
@@ -890,23 +890,23 @@
         </is>
       </c>
       <c r="C10" s="2">
-        <f>COUNTIF(B$19:B$38,$B10)</f>
+        <f>COUNTIF(B$19:B$50,$B10)</f>
         <v/>
       </c>
       <c r="D10" s="2">
-        <f>COUNTIF(C$19:C$38,$B10)</f>
+        <f>COUNTIF(C$19:C$50,$B10)</f>
         <v/>
       </c>
       <c r="E10" s="2">
-        <f>COUNTIF(D$19:D$38,$B10)</f>
+        <f>COUNTIF(D$19:D$50,$B10)</f>
         <v/>
       </c>
       <c r="F10" s="2">
-        <f>COUNTIF(E$19:E$38,$B10)</f>
+        <f>COUNTIF(E$19:E$50,$B10)</f>
         <v/>
       </c>
       <c r="G10" s="2">
-        <f>COUNTIF(F$19:F$38,$B10)</f>
+        <f>COUNTIF(F$19:F$50,$B10)</f>
         <v/>
       </c>
       <c r="I10" s="1" t="inlineStr">
@@ -958,23 +958,23 @@
         </is>
       </c>
       <c r="C11" s="2">
-        <f>COUNTIF(B$19:B$38,$B11)</f>
+        <f>COUNTIF(B$19:B$50,$B11)</f>
         <v/>
       </c>
       <c r="D11" s="2">
-        <f>COUNTIF(C$19:C$38,$B11)</f>
+        <f>COUNTIF(C$19:C$50,$B11)</f>
         <v/>
       </c>
       <c r="E11" s="2">
-        <f>COUNTIF(D$19:D$38,$B11)</f>
+        <f>COUNTIF(D$19:D$50,$B11)</f>
         <v/>
       </c>
       <c r="F11" s="2">
-        <f>COUNTIF(E$19:E$38,$B11)</f>
+        <f>COUNTIF(E$19:E$50,$B11)</f>
         <v/>
       </c>
       <c r="G11" s="2">
-        <f>COUNTIF(F$19:F$38,$B11)</f>
+        <f>COUNTIF(F$19:F$50,$B11)</f>
         <v/>
       </c>
       <c r="I11" s="1" t="inlineStr">
@@ -1026,23 +1026,23 @@
         </is>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIF(B$19:B$38,$B12)</f>
+        <f>COUNTIF(B$19:B$50,$B12)</f>
         <v/>
       </c>
       <c r="D12" s="2">
-        <f>COUNTIF(C$19:C$38,$B12)</f>
+        <f>COUNTIF(C$19:C$50,$B12)</f>
         <v/>
       </c>
       <c r="E12" s="2">
-        <f>COUNTIF(D$19:D$38,$B12)</f>
+        <f>COUNTIF(D$19:D$50,$B12)</f>
         <v/>
       </c>
       <c r="F12" s="2">
-        <f>COUNTIF(E$19:E$38,$B12)</f>
+        <f>COUNTIF(E$19:E$50,$B12)</f>
         <v/>
       </c>
       <c r="G12" s="2">
-        <f>COUNTIF(F$19:F$38,$B12)</f>
+        <f>COUNTIF(F$19:F$50,$B12)</f>
         <v/>
       </c>
       <c r="I12" s="1" t="inlineStr">
@@ -1094,23 +1094,23 @@
         </is>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIF(B$19:B$38,$B13)</f>
+        <f>COUNTIF(B$19:B$50,$B13)</f>
         <v/>
       </c>
       <c r="D13" s="2">
-        <f>COUNTIF(C$19:C$38,$B13)</f>
+        <f>COUNTIF(C$19:C$50,$B13)</f>
         <v/>
       </c>
       <c r="E13" s="2">
-        <f>COUNTIF(D$19:D$38,$B13)</f>
+        <f>COUNTIF(D$19:D$50,$B13)</f>
         <v/>
       </c>
       <c r="F13" s="2">
-        <f>COUNTIF(E$19:E$38,$B13)</f>
+        <f>COUNTIF(E$19:E$50,$B13)</f>
         <v/>
       </c>
       <c r="G13" s="2">
-        <f>COUNTIF(F$19:F$38,$B13)</f>
+        <f>COUNTIF(F$19:F$50,$B13)</f>
         <v/>
       </c>
       <c r="I13" s="1" t="inlineStr">
@@ -1296,22 +1296,22 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Wolf</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Wild</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1359,29 +1359,29 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>J</t>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Wild</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>J</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>Q</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>King</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Queen</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1407,20 +1407,20 @@
           <t>J</t>
         </is>
       </c>
-      <c r="P20" s="5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q20" s="5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R20" s="5" t="n">
-        <v>0.7</v>
+      <c r="P20" s="6" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="Q20" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>2.85</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1430,17 +1430,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>King</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>K</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Q</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1466,40 +1466,40 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="P21" s="5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="Q21" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="R21" s="5" t="n">
-        <v>0.85</v>
+      <c r="P21" s="6" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>4.56</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+          <t>King</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Wild</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>Q</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>King</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Wolf</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1525,40 +1525,40 @@
           <t>K</t>
         </is>
       </c>
-      <c r="P22" s="5" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Q22" s="5" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="R22" s="5" t="n">
-        <v>1.25</v>
+      <c r="P22" s="6" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="Q22" s="6" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>7.13</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>Wolf</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>King</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1584,30 +1584,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="P23" s="5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q23" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="R23" s="5" t="n">
-        <v>1.7</v>
+      <c r="P23" s="6" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="Q23" s="6" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>11.4</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Queen</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1643,30 +1643,30 @@
           <t>Wolf</t>
         </is>
       </c>
-      <c r="P24" s="5" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="Q24" s="5" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="R24" s="5" t="n">
-        <v>2.55</v>
+      <c r="P24" s="6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="Q24" s="6" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="R24" s="6" t="n">
+        <v>18.53</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wolf</t>
+          <t>J</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>J</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -1702,25 +1702,25 @@
           <t>Queen</t>
         </is>
       </c>
-      <c r="P25" s="5" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Q25" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="R25" s="5" t="n">
-        <v>4.25</v>
+      <c r="P25" s="6" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="Q25" s="6" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>28.51</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>King</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1730,12 +1730,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>Wolf</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -1761,20 +1761,20 @@
           <t>King</t>
         </is>
       </c>
-      <c r="P26" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Q26" s="5" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="R26" s="5" t="n">
-        <v>8.4</v>
+      <c r="P26" s="6" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="Q26" s="6" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>42.76</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1784,17 +1784,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Wolf</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>K</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -1820,40 +1820,40 @@
           <t>Wild</t>
         </is>
       </c>
-      <c r="P27" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q27" s="5" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="R27" s="5" t="n">
-        <v>12.5</v>
+      <c r="P27" s="6" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>71.27</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>Wolf</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>Wolf</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -1878,46 +1878,28 @@
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
           <t>King</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Wolf</t>
-        </is>
-      </c>
-      <c r="H29" t="n">
-        <v>10</v>
-      </c>
-      <c r="I29" t="n">
-        <v>2</v>
-      </c>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" t="n">
-        <v>1</v>
-      </c>
-      <c r="M29" t="n">
-        <v>2</v>
+          <t>J</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1928,41 +1910,23 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Wolf</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>King</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>11</v>
-      </c>
-      <c r="I30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>1</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="n">
-        <v>1</v>
+          <t>Queen</t>
+        </is>
       </c>
       <c r="O30" s="3" t="inlineStr"/>
       <c r="P30" s="3" t="inlineStr">
@@ -1979,57 +1943,39 @@
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Wolf</t>
-        </is>
-      </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="H31" t="n">
-        <v>12</v>
-      </c>
-      <c r="I31" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" t="n">
-        <v>2</v>
-      </c>
-      <c r="M31" t="n">
-        <v>1</v>
-      </c>
       <c r="O31" s="1" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="P31" s="6">
+      <c r="P31" s="7">
         <f>SUM(R6:R13)*$E$3</f>
         <v/>
       </c>
-      <c r="Q31" s="5">
+      <c r="Q31" s="6">
         <f>P31*100</f>
         <v/>
       </c>
@@ -2037,57 +1983,39 @@
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Wolf</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>13</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="n">
-        <v>1</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="n">
-        <v>1</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0</v>
-      </c>
       <c r="O32" s="1" t="inlineStr">
         <is>
           <t>Wild Pay</t>
         </is>
       </c>
-      <c r="P32" s="6">
-        <f>L45</f>
-        <v/>
-      </c>
-      <c r="Q32" s="5">
+      <c r="P32" s="7">
+        <f>L49</f>
+        <v/>
+      </c>
+      <c r="Q32" s="6">
         <f>P32*100</f>
         <v/>
       </c>
@@ -2095,57 +2023,39 @@
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>King</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>King</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Wild</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>14</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2</v>
-      </c>
-      <c r="J33" t="n">
-        <v>1</v>
-      </c>
-      <c r="K33" t="n">
-        <v>2</v>
-      </c>
-      <c r="L33" t="n">
-        <v>1</v>
-      </c>
-      <c r="M33" t="n">
-        <v>2</v>
+          <t>Q</t>
+        </is>
       </c>
       <c r="O33" s="1" t="inlineStr">
         <is>
           <t>Bonus</t>
         </is>
       </c>
-      <c r="P33" s="6">
-        <f>O52</f>
-        <v/>
-      </c>
-      <c r="Q33" s="5">
+      <c r="P33" s="7">
+        <f>O56</f>
+        <v/>
+      </c>
+      <c r="Q33" s="6">
         <f>P33*100</f>
         <v/>
       </c>
@@ -2153,46 +2063,28 @@
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>King</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Wolf</t>
-        </is>
-      </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>King</t>
         </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Wild</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
-        <v>15</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
-      <c r="L34" t="n">
-        <v>2</v>
-      </c>
-      <c r="M34" t="n">
-        <v>2</v>
       </c>
       <c r="O34" s="8" t="inlineStr">
         <is>
@@ -2211,101 +2103,65 @@
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>Queen</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Wild</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="H35" t="n">
-        <v>16</v>
-      </c>
-      <c r="I35" t="n">
-        <v>2</v>
-      </c>
-      <c r="J35" t="n">
-        <v>2</v>
-      </c>
-      <c r="K35" t="n">
-        <v>1</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Wild</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="H36" t="n">
-        <v>17</v>
-      </c>
-      <c r="I36" t="n">
-        <v>1</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" t="n">
-        <v>1</v>
-      </c>
-      <c r="M36" t="n">
-        <v>2</v>
+          <t>A</t>
+        </is>
       </c>
       <c r="O36" s="1" t="inlineStr">
         <is>
           <t>Hit Rate</t>
         </is>
       </c>
-      <c r="P36" s="6" t="n">
-        <v>0.466446875</v>
-      </c>
-      <c r="Q36" s="5">
+      <c r="P36" s="7" t="n">
+        <v>0.3065</v>
+      </c>
+      <c r="Q36" s="6">
         <f>P36*100</f>
         <v/>
       </c>
@@ -2313,7 +2169,7 @@
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2323,7 +2179,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2333,26 +2189,8 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Wolf</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>18</v>
-      </c>
-      <c r="I37" t="n">
-        <v>1</v>
-      </c>
-      <c r="J37" t="n">
-        <v>2</v>
-      </c>
-      <c r="K37" t="n">
-        <v>2</v>
-      </c>
-      <c r="L37" t="n">
-        <v>1</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
+          <t>Queen</t>
+        </is>
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
@@ -2363,577 +2201,871 @@
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
           <t>Wolf</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>Wild</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>Wild</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>King</t>
         </is>
       </c>
-      <c r="H38" t="n">
-        <v>19</v>
-      </c>
-      <c r="I38" t="n">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>WILD PAY (Wild on grid)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Wilds</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>P(k wilds)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Combinations</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Wild Pay (xTBet)</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Wild Pay RTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>3</v>
+      </c>
+      <c r="I46" s="4">
+        <f>O16</f>
+        <v/>
+      </c>
+      <c r="J46" s="6">
+        <f>I46*$F$3</f>
+        <v/>
+      </c>
+      <c r="K46" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L46" s="7">
+        <f>I46*K46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>4</v>
+      </c>
+      <c r="I47" s="4">
+        <f>P16</f>
+        <v/>
+      </c>
+      <c r="J47" s="6">
+        <f>I47*$F$3</f>
+        <v/>
+      </c>
+      <c r="K47" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="L47" s="7">
+        <f>I47*K47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>5</v>
+      </c>
+      <c r="I48" s="4">
+        <f>Q16</f>
+        <v/>
+      </c>
+      <c r="J48" s="6">
+        <f>I48*$F$3</f>
+        <v/>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="L48" s="7">
+        <f>I48*K48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>Total Wild Pay</t>
+        </is>
+      </c>
+      <c r="J49" s="6">
+        <f>SUM(J46:J48)</f>
+        <v/>
+      </c>
+      <c r="L49" s="7">
+        <f>SUM(L46:L48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="H51" s="12" t="inlineStr">
+        <is>
+          <t>BONUS CHESTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Wilds</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Prizes (xTBet)</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Pool</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>Skulls</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>E[picks]</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>EV bonus (xTBet)</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>Bonus RTP</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>Wild Pay</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
+        <is>
+          <t>Bonus EV</t>
+        </is>
+      </c>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>Total EV</t>
+        </is>
+      </c>
+      <c r="T52" s="3" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="U52" s="3" t="inlineStr">
+        <is>
+          <t>Match?</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="H53" t="n">
         <v>0</v>
       </c>
-      <c r="J38" t="n">
+      <c r="I53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>25, 75, 125</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>225</v>
+      </c>
+      <c r="L53" t="n">
+        <v>2</v>
+      </c>
+      <c r="M53" s="6">
+        <f>(5-L53)/(L53+1)</f>
+        <v/>
+      </c>
+      <c r="N53" s="6">
+        <f>K53/(L53+1)</f>
+        <v/>
+      </c>
+      <c r="O53" s="7">
+        <f>I46*N53</f>
+        <v/>
+      </c>
+      <c r="Q53" s="6">
+        <f>K46</f>
+        <v/>
+      </c>
+      <c r="R53" s="6">
+        <f>N53</f>
+        <v/>
+      </c>
+      <c r="S53" s="6">
+        <f>Q53+R53</f>
+        <v/>
+      </c>
+      <c r="T53" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="U53">
+        <f>IF(ABS(S53-T53)&lt;0.01,"OK","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="H54" t="n">
         <v>1</v>
       </c>
-      <c r="K38" t="n">
+      <c r="I54" t="n">
+        <v>4</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>30, 60, 90, 120</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>300</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" s="6">
+        <f>(5-L54)/(L54+1)</f>
+        <v/>
+      </c>
+      <c r="N54" s="6">
+        <f>K54/(L54+1)</f>
+        <v/>
+      </c>
+      <c r="O54" s="7">
+        <f>I47*N54</f>
+        <v/>
+      </c>
+      <c r="Q54" s="6">
+        <f>K47</f>
+        <v/>
+      </c>
+      <c r="R54" s="6">
+        <f>N54</f>
+        <v/>
+      </c>
+      <c r="S54" s="6">
+        <f>Q54+R54</f>
+        <v/>
+      </c>
+      <c r="T54" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="U54">
+        <f>IF(ABS(S54-T54)&lt;0.01,"OK","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="H55" t="n">
         <v>2</v>
       </c>
-      <c r="L38" t="n">
-        <v>2</v>
-      </c>
-      <c r="M38" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="H40" s="12" t="inlineStr">
-        <is>
-          <t>WILD PAY (Wild en grid)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Wilds</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>P(k wilds)</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>Combinaciones</t>
-        </is>
-      </c>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t>Wild Pay (xTBet)</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="inlineStr">
-        <is>
-          <t>Wild Pay RTP</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="H42" t="n">
-        <v>3</v>
-      </c>
-      <c r="I42" s="4">
-        <f>O16</f>
-        <v/>
-      </c>
-      <c r="J42" s="5">
-        <f>I42*$F$3</f>
-        <v/>
-      </c>
-      <c r="K42" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L42" s="6">
-        <f>I42*K42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="H43" t="n">
-        <v>4</v>
-      </c>
-      <c r="I43" s="4">
-        <f>P16</f>
-        <v/>
-      </c>
-      <c r="J43" s="5">
-        <f>I43*$F$3</f>
-        <v/>
-      </c>
-      <c r="K43" s="5" t="n">
+      <c r="I55" t="n">
         <v>5</v>
       </c>
-      <c r="L43" s="6">
-        <f>I43*K43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="H44" t="n">
-        <v>5</v>
-      </c>
-      <c r="I44" s="4">
-        <f>Q16</f>
-        <v/>
-      </c>
-      <c r="J44" s="5">
-        <f>I44*$F$3</f>
-        <v/>
-      </c>
-      <c r="K44" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="L44" s="6">
-        <f>I44*K44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="H45" s="1" t="inlineStr">
-        <is>
-          <t>Total Wild Pay</t>
-        </is>
-      </c>
-      <c r="J45" s="5">
-        <f>SUM(J42:J44)</f>
-        <v/>
-      </c>
-      <c r="L45" s="6">
-        <f>SUM(L42:L44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="H47" s="12" t="inlineStr">
-        <is>
-          <t>BONUS COFRES</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="H48" s="3" t="inlineStr">
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>20, 40, 60, 80, 100</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>300</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="6">
+        <f>(5-L55)/(L55+1)</f>
+        <v/>
+      </c>
+      <c r="N55" s="6">
+        <f>K55/(L55+1)</f>
+        <v/>
+      </c>
+      <c r="O55" s="7">
+        <f>I48*N55</f>
+        <v/>
+      </c>
+      <c r="Q55" s="6">
+        <f>K48</f>
+        <v/>
+      </c>
+      <c r="R55" s="6">
+        <f>N55</f>
+        <v/>
+      </c>
+      <c r="S55" s="6">
+        <f>Q55+R55</f>
+        <v/>
+      </c>
+      <c r="T55" s="6" t="n">
+        <v>383</v>
+      </c>
+      <c r="U55">
+        <f>IF(ABS(S55-T55)&lt;0.01,"OK","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>Total Bonus</t>
+        </is>
+      </c>
+      <c r="O56" s="7">
+        <f>SUM(O53:O55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>BUY BONUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="I48" s="3" t="inlineStr">
-        <is>
-          <t>Wilds</t>
-        </is>
-      </c>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t>Prizes (xTBet)</t>
-        </is>
-      </c>
-      <c r="K48" s="3" t="inlineStr">
-        <is>
-          <t>Pool</t>
-        </is>
-      </c>
-      <c r="L48" s="3" t="inlineStr">
-        <is>
-          <t>Skulls</t>
-        </is>
-      </c>
-      <c r="M48" s="3" t="inlineStr">
-        <is>
-          <t>E[picks]</t>
-        </is>
-      </c>
-      <c r="N48" s="3" t="inlineStr">
-        <is>
-          <t>EV bonus (xTBet)</t>
-        </is>
-      </c>
-      <c r="O48" s="3" t="inlineStr">
-        <is>
-          <t>Bonus RTP</t>
-        </is>
-      </c>
-      <c r="Q48" s="3" t="inlineStr">
-        <is>
-          <t>Wild Pay</t>
-        </is>
-      </c>
-      <c r="R48" s="3" t="inlineStr">
-        <is>
-          <t>Bonus EV</t>
-        </is>
-      </c>
-      <c r="S48" s="3" t="inlineStr">
-        <is>
-          <t>Total EV</t>
-        </is>
-      </c>
-      <c r="T48" s="3" t="inlineStr">
-        <is>
-          <t>Old EV</t>
-        </is>
-      </c>
-      <c r="U48" s="3" t="inlineStr">
-        <is>
-          <t>Match?</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="H49" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" t="n">
-        <v>3</v>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>8, 18, 28</t>
-        </is>
-      </c>
-      <c r="K49" t="n">
-        <v>54</v>
-      </c>
-      <c r="L49" t="n">
-        <v>2</v>
-      </c>
-      <c r="M49" s="5">
-        <f>(5-L49)/(L49+1)</f>
-        <v/>
-      </c>
-      <c r="N49" s="5">
-        <f>K49/(L49+1)</f>
-        <v/>
-      </c>
-      <c r="O49" s="6">
-        <f>I42*N49</f>
-        <v/>
-      </c>
-      <c r="Q49" s="5">
-        <f>K42</f>
-        <v/>
-      </c>
-      <c r="R49" s="5">
-        <f>N49</f>
-        <v/>
-      </c>
-      <c r="S49" s="5">
-        <f>Q49+R49</f>
-        <v/>
-      </c>
-      <c r="T49" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="U49">
-        <f>IF(ABS(S49-T49)&lt;0.01,"OK","FAIL")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="H50" t="n">
-        <v>1</v>
-      </c>
-      <c r="I50" t="n">
-        <v>4</v>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>8, 15, 20, 27</t>
-        </is>
-      </c>
-      <c r="K50" t="n">
-        <v>70</v>
-      </c>
-      <c r="L50" t="n">
-        <v>1</v>
-      </c>
-      <c r="M50" s="5">
-        <f>(5-L50)/(L50+1)</f>
-        <v/>
-      </c>
-      <c r="N50" s="5">
-        <f>K50/(L50+1)</f>
-        <v/>
-      </c>
-      <c r="O50" s="6">
-        <f>I43*N50</f>
-        <v/>
-      </c>
-      <c r="Q50" s="5">
-        <f>K43</f>
-        <v/>
-      </c>
-      <c r="R50" s="5">
-        <f>N50</f>
-        <v/>
-      </c>
-      <c r="S50" s="5">
-        <f>Q50+R50</f>
-        <v/>
-      </c>
-      <c r="T50" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="U50">
-        <f>IF(ABS(S50-T50)&lt;0.01,"OK","FAIL")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="H51" t="n">
-        <v>2</v>
-      </c>
-      <c r="I51" t="n">
-        <v>5</v>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>8, 10, 15, 20, 27</t>
-        </is>
-      </c>
-      <c r="K51" t="n">
-        <v>80</v>
-      </c>
-      <c r="L51" t="n">
-        <v>0</v>
-      </c>
-      <c r="M51" s="5">
-        <f>(5-L51)/(L51+1)</f>
-        <v/>
-      </c>
-      <c r="N51" s="5">
-        <f>K51/(L51+1)</f>
-        <v/>
-      </c>
-      <c r="O51" s="6">
-        <f>I44*N51</f>
-        <v/>
-      </c>
-      <c r="Q51" s="5">
-        <f>K44</f>
-        <v/>
-      </c>
-      <c r="R51" s="5">
-        <f>N51</f>
-        <v/>
-      </c>
-      <c r="S51" s="5">
-        <f>Q51+R51</f>
-        <v/>
-      </c>
-      <c r="T51" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="U51">
-        <f>IF(ABS(S51-T51)&lt;0.01,"OK","FAIL")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="H52" s="1" t="inlineStr">
-        <is>
-          <t>Total Bonus</t>
-        </is>
-      </c>
-      <c r="O52" s="6">
-        <f>SUM(O49:O51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="H54" s="12" t="inlineStr">
-        <is>
-          <t>BUY BONUS</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>Simula</t>
-        </is>
-      </c>
-      <c r="J55" s="3" t="inlineStr">
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Simulates</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
         <is>
           <t>EV total (xTBet)</t>
         </is>
       </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
-          <t>Precio (xTBet)</t>
-        </is>
-      </c>
-      <c r="L55" s="3" t="inlineStr">
-        <is>
-          <t>RTP Buy</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="H56" t="inlineStr">
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Price (xTBet)</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>Buy RTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>3 Wilds</t>
         </is>
       </c>
-      <c r="J56" s="5">
-        <f>S49</f>
-        <v/>
-      </c>
-      <c r="K56" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="L56" s="6">
-        <f>J56/K56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="H57" t="inlineStr">
+      <c r="J60" s="6">
+        <f>S53</f>
+        <v/>
+      </c>
+      <c r="K60" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="L60" s="7">
+        <f>J60/K60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>4 Wilds</t>
         </is>
       </c>
-      <c r="J57" s="5">
-        <f>S50</f>
-        <v/>
-      </c>
-      <c r="K57" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="L57" s="6">
-        <f>J57/K57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Tier 3</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>5 Wilds</t>
-        </is>
-      </c>
-      <c r="J58" s="5">
-        <f>S51</f>
-        <v/>
-      </c>
-      <c r="K58" s="5" t="n">
-        <v>105</v>
-      </c>
-      <c r="L58" s="6">
-        <f>J58/K58</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="H60" s="12" t="inlineStr">
-        <is>
-          <t>VERIFICACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>Resultado</t>
-        </is>
+      <c r="J61" s="6">
+        <f>S54</f>
+        <v/>
+      </c>
+      <c r="K61" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="L61" s="7">
+        <f>J61/K61</f>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="H62" t="inlineStr">
         <is>
-          <t>RTP total = 96.12%?</t>
-        </is>
-      </c>
-      <c r="I62" s="1">
-        <f>IF(ABS(P34-0.961232)&lt;0.0001,"PASS","FAIL")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>WildPay+Bonus = 58.13%?</t>
-        </is>
-      </c>
-      <c r="I63" s="1">
-        <f>IF(ABS(P32+P33-0.581344)&lt;0.0001,"PASS","FAIL")</f>
+          <t>Tier 3</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>5 Wilds</t>
+        </is>
+      </c>
+      <c r="J62" s="6">
+        <f>S55</f>
+        <v/>
+      </c>
+      <c r="K62" s="6" t="n">
+        <v>403</v>
+      </c>
+      <c r="L62" s="7">
+        <f>J62/K62</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>Line RTP = 37.99%?</t>
-        </is>
-      </c>
-      <c r="I64" s="1">
-        <f>IF(ABS(P31-0.379888)&lt;0.0001,"PASS","FAIL")</f>
-        <v/>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>VERIFICATIONS</t>
+        </is>
       </c>
     </row>
     <row r="65">
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>EV 3W = 20?</t>
-        </is>
-      </c>
-      <c r="I65" s="1">
-        <f>IF(ABS(S49-T49)&lt;0.01,"PASS","FAIL")</f>
-        <v/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="H66" t="inlineStr">
         <is>
-          <t>EV 4W = 40?</t>
+          <t>RTP total ~ 96.14%?</t>
         </is>
       </c>
       <c r="I66" s="1">
-        <f>IF(ABS(S50-T50)&lt;0.01,"PASS","FAIL")</f>
+        <f>IF(ABS(P34-0.9614)&lt;0.002,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="H67" t="inlineStr">
         <is>
-          <t>EV 5W = 100?</t>
+          <t>WildPay+Bonus ~ 62.43%?</t>
         </is>
       </c>
       <c r="I67" s="1">
-        <f>IF(ABS(S51-T51)&lt;0.01,"PASS","FAIL")</f>
+        <f>IF(ABS(P32+P33-0.6243)&lt;0.002,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Line RTP ~ 33.71%?</t>
+        </is>
+      </c>
+      <c r="I68" s="1">
+        <f>IF(ABS(P31-0.3371)&lt;0.002,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>EV 3W = 83?</t>
+        </is>
+      </c>
+      <c r="I69" s="1">
+        <f>IF(ABS(S53-T53)&lt;0.01,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>EV 4W = 171?</t>
+        </is>
+      </c>
+      <c r="I70" s="1">
+        <f>IF(ABS(S54-T54)&lt;0.01,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>EV 5W = 383?</t>
+        </is>
+      </c>
+      <c r="I71" s="1">
+        <f>IF(ABS(S55-T55)&lt;0.01,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
remove wild pay, inflate T0 bonus pool, rework bonus entry presentation
- Remove wild pay entirely (3W=0, 4W=0, 5W=0) — wilds only trigger bonus
- T0 bonus pool changed from [25,75,125] to [30,75,150] (pool=255, EV=85x)
- Buy bonus prices updated: 88→89 (T1), 180→158 (T2)
- Win presentation reordered for bonus: wilds first → total → lines → loop
- Wild step plays bonusRoundAnnounce voice (every 2 cycles if no paylines)
- Balance updates deferred to celebration start instead of reel stop
- Bonus return celebration shows only bonus win (no longer adds entry win)
- RTP verified at 96.70% (analytical + 10M MC simulation)
</commit_message>
<xml_diff>
--- a/docs/total-bet-model-rtp.xlsx
+++ b/docs/total-bet-model-rtp.xlsx
@@ -2482,7 +2482,7 @@
         <v/>
       </c>
       <c r="K46" s="6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L46" s="7">
         <f>I46*K46</f>
@@ -2527,7 +2527,7 @@
         <v/>
       </c>
       <c r="K47" s="6" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="L47" s="7">
         <f>I47*K47</f>
@@ -2572,7 +2572,7 @@
         <v/>
       </c>
       <c r="K48" s="6" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="L48" s="7">
         <f>I48*K48</f>
@@ -2729,11 +2729,11 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>25, 75, 125</t>
+          <t>30, 75, 150</t>
         </is>
       </c>
       <c r="K53" t="n">
-        <v>225</v>
+        <v>255</v>
       </c>
       <c r="L53" t="n">
         <v>2</v>

</xml_diff>